<commit_message>
feat: ajuste da função de remoção de duplicados
</commit_message>
<xml_diff>
--- a/data_processed/metricas_todas_abas.xlsx
+++ b/data_processed/metricas_todas_abas.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,148 +454,178 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BISCOITO</t>
+          <t>BAGEL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3090</v>
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>R$ 3.223,00</t>
+          <t>R$ 2,00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BOLO</t>
+          <t>BISCOITO</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3329</v>
+        <v>3090</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>R$ 10.395,00</t>
+          <t>R$ 3.223,00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAFÉ</t>
+          <t>BOLO</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3368</v>
+        <v>3333</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>R$ 7.062,00</t>
+          <t>R$ 10.407,00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CHÁ</t>
+          <t>CAFÉ</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3154</v>
+        <v>3368</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>R$ 4.951,50</t>
+          <t>R$ 7.062,00</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EXPRESSO</t>
+          <t>CHÁ</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>3157</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>R$ 2,50</t>
+          <t>R$ 4.956,00</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>LATTE</t>
+          <t>EXPRESSO</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>R$ 7,00</t>
+          <t>R$ 2,50</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SALADA</t>
+          <t>LATTE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3310</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>R$ 17.320,00</t>
+          <t>R$ 14,00</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SANDUICHE</t>
+          <t>MUFFIN</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3245</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>R$ 13.664,00</t>
+          <t>R$ 13,00</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SUCO</t>
+          <t>SALADA</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3373</v>
+        <v>3310</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>R$ 10.509,00</t>
+          <t>R$ 17.320,00</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>SANDUICHE</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3249</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>R$ 13.680,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SUCO</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3373</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>R$ 10.509,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>VITAMINA</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B13" t="n">
         <v>3221</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>R$ 13.320,00</t>
         </is>
@@ -635,7 +665,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 88,961.50</t>
+          <t>R$ 89,016.00</t>
         </is>
       </c>
     </row>
@@ -678,11 +708,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 20.383,50</t>
+          <t>R$ 20.385,50</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2291</v>
+        <v>2292</v>
       </c>
     </row>
     <row r="3">
@@ -693,11 +723,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 20.436,50</t>
+          <t>R$ 20.443,50</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2275</v>
+        <v>2276</v>
       </c>
     </row>
     <row r="4">
@@ -708,11 +738,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R$ 20.366,50</t>
+          <t>R$ 20.412,00</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2258</v>
+        <v>2263</v>
       </c>
     </row>
   </sheetData>
@@ -749,7 +779,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 8.89</t>
+          <t>R$ 8.90</t>
         </is>
       </c>
     </row>
@@ -828,11 +858,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 26.497,00</t>
+          <t>R$ 26.513,00</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3024</v>
+        <v>3027</v>
       </c>
     </row>
     <row r="3">
@@ -843,11 +873,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 27.127,00</t>
+          <t>R$ 27.149,50</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3017</v>
+        <v>3020</v>
       </c>
     </row>
   </sheetData>
@@ -884,7 +914,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>R$ 12.137,50</t>
+          <t>R$ 12.139,50</t>
         </is>
       </c>
     </row>
@@ -896,7 +926,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>R$ 12.030,50</t>
+          <t>R$ 12.048,50</t>
         </is>
       </c>
     </row>
@@ -908,7 +938,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>R$ 11.623,50</t>
+          <t>R$ 11.630,50</t>
         </is>
       </c>
     </row>
@@ -932,7 +962,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R$ 12.317,50</t>
+          <t>R$ 12.324,50</t>
         </is>
       </c>
     </row>
@@ -944,7 +974,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R$ 12.007,50</t>
+          <t>R$ 12.023,50</t>
         </is>
       </c>
     </row>
@@ -956,7 +986,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R$ 12.285,50</t>
+          <t>R$ 12.290,00</t>
         </is>
       </c>
     </row>

</xml_diff>